<commit_message>
Updated LHJ Population Data File (date updated: 2025.10.21) with newest DOF P3 Vintage 2025 (released 2025.09.30)
</commit_message>
<xml_diff>
--- a/LHJ Data/finalPopData/Data-Dictionary.xlsx
+++ b/LHJ Data/finalPopData/Data-Dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\FusionData\Population Task Force\LHJ Data\finalPopData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2F97E1-19FA-42F1-8BFE-0A14776DEC6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF223ADD-EB60-4113-9DE4-5DB3B65B0D60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15315" yWindow="3270" windowWidth="26520" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Column</t>
   </si>
@@ -64,15 +64,9 @@
     <t>Population estimates</t>
   </si>
   <si>
-    <t>LHJ Population dataset last updated May 21, 2025</t>
-  </si>
-  <si>
     <t>Data Sources:</t>
   </si>
   <si>
-    <t>DOF P3 Vintage 2025 (released 2025.04.25)</t>
-  </si>
-  <si>
     <t>DOF Annual Intercensal 2010-2020 (released 2025.01.29) and 2000-2010 (released 2013.03.19)</t>
   </si>
   <si>
@@ -83,6 +77,18 @@
   </si>
   <si>
     <t>Census Decennial 2000, 2010, and 2020</t>
+  </si>
+  <si>
+    <t>Recommended Citation:</t>
+  </si>
+  <si>
+    <t>LHJ Population dataset last updated October 21, 2025</t>
+  </si>
+  <si>
+    <t>DOF P3 Vintage 2025 (released 2025.09.30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">California Department of Public Health, Population Task Force. (Published October 21, 2025). Local Health Jurisdiction Population Estimates by Age by Race and Ethnicity by Sex [Data set]. https://github.com/mcSamuelDataSci/CDPH-LHJ-Population-Task-Force/blob/main/LHJ%20Data/finalPopData/lhj-pop-ars-2000-cy.csv </t>
   </si>
 </sst>
 </file>
@@ -450,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -515,37 +521,47 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>